<commit_message>
updated Project Kaskan - checking sources
</commit_message>
<xml_diff>
--- a/____Unpublished__ProjectKaskan/Rachael_Robinson_dissertation_file_copies/Brains data for animals/Results Rachael krubitzer_kaas_1993_marmoset and owl monkey.xlsx
+++ b/____Unpublished__ProjectKaskan/Rachael_Robinson_dissertation_file_copies/Brains data for animals/Results Rachael krubitzer_kaas_1993_marmoset and owl monkey.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23801"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rachael\OneDrive\Documents\PS30094 Dissertation\Brain area data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alleninstitute.sharepoint.com/sites/MammalianM1/Shared Documents/General/Species/Evo-M1-Trait-Data/____Unpublished__ProjectKaskan/Rachael_Robinson_dissertation_file_copies/Brains data for animals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2A13EB3-AB17-4F2B-99C0-57367206C197}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{F2A13EB3-AB17-4F2B-99C0-57367206C197}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{516E7006-3DF3-5D42-8550-DBF1E55EE6EA}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="4" xr2:uid="{FCAE0888-F5B4-4644-A0E8-01483E3D1D7F}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="33460" windowHeight="18200" activeTab="1" xr2:uid="{FCAE0888-F5B4-4644-A0E8-01483E3D1D7F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -310,9 +310,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -350,7 +350,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -456,7 +456,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -598,7 +598,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -607,12 +607,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83987BEF-DFC0-4F03-8D3B-10A20AF96867}">
   <dimension ref="A1:R23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="15" max="15" width="15.54296875" customWidth="1"/>
+    <col min="13" max="13" width="8.83203125" customWidth="1"/>
+    <col min="15" max="15" width="15.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -656,7 +657,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -704,7 +705,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -756,7 +757,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -801,7 +802,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -840,7 +841,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -879,7 +880,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -918,7 +919,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>4</v>
       </c>
@@ -957,7 +958,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>7</v>
       </c>
@@ -993,7 +994,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>8</v>
       </c>
@@ -1029,7 +1030,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>9</v>
       </c>
@@ -1065,7 +1066,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>10</v>
       </c>
@@ -1101,7 +1102,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>11</v>
       </c>
@@ -1137,7 +1138,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14" s="2"/>
       <c r="J14">
         <v>1</v>
@@ -1149,7 +1150,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>12</v>
       </c>
@@ -1185,7 +1186,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
         <v>2</v>
       </c>
@@ -1221,7 +1222,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>13</v>
       </c>
@@ -1257,7 +1258,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>14</v>
       </c>
@@ -1293,7 +1294,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
         <v>3</v>
       </c>
@@ -1329,7 +1330,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
         <v>1</v>
       </c>
@@ -1356,7 +1357,7 @@
         <v>29.2545</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
       <c r="P23">
         <f>P22^2</f>
         <v>855.82577025000001</v>
@@ -1370,14 +1371,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90D4BE22-14BE-4BE5-9443-031264EB9F9A}">
   <dimension ref="A1:R22"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="13" max="13" width="8.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>1</v>
       </c>
@@ -1418,7 +1422,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1466,7 +1470,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2</v>
       </c>
@@ -1518,7 +1522,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>3</v>
       </c>
@@ -1563,7 +1567,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>4</v>
       </c>
@@ -1599,7 +1603,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>5</v>
       </c>
@@ -1635,7 +1639,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>6</v>
       </c>
@@ -1671,7 +1675,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>7</v>
       </c>
@@ -1707,7 +1711,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>8</v>
       </c>
@@ -1743,7 +1747,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>9</v>
       </c>
@@ -1779,7 +1783,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>10</v>
       </c>
@@ -1815,7 +1819,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>11</v>
       </c>
@@ -1851,7 +1855,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>12</v>
       </c>
@@ -1887,7 +1891,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>13</v>
       </c>
@@ -1923,7 +1927,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>14</v>
       </c>
@@ -1959,7 +1963,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>15</v>
       </c>
@@ -1995,7 +1999,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>16</v>
       </c>
@@ -2031,7 +2035,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>17</v>
       </c>
@@ -2067,7 +2071,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>18</v>
       </c>
@@ -2103,7 +2107,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>19</v>
       </c>
@@ -2139,7 +2143,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>20</v>
       </c>
@@ -2183,14 +2187,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A40B589-69DA-4949-86B1-E20E13C270B9}">
   <dimension ref="A1:R22"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>1</v>
       </c>
@@ -2231,7 +2235,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2279,7 +2283,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2</v>
       </c>
@@ -2331,7 +2335,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>3</v>
       </c>
@@ -2376,7 +2380,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>4</v>
       </c>
@@ -2412,7 +2416,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>5</v>
       </c>
@@ -2448,7 +2452,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>6</v>
       </c>
@@ -2484,7 +2488,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="J9" t="s">
         <v>35</v>
       </c>
@@ -2499,7 +2503,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>7</v>
       </c>
@@ -2535,7 +2539,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>8</v>
       </c>
@@ -2571,7 +2575,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>9</v>
       </c>
@@ -2607,7 +2611,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>10</v>
       </c>
@@ -2643,7 +2647,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="J14">
         <v>1</v>
       </c>
@@ -2658,7 +2662,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>11</v>
       </c>
@@ -2694,7 +2698,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="J16" t="s">
         <v>52</v>
       </c>
@@ -2702,7 +2706,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="10:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="10:11" x14ac:dyDescent="0.2">
       <c r="J17" t="s">
         <v>39</v>
       </c>
@@ -2710,7 +2714,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="10:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="10:11" x14ac:dyDescent="0.2">
       <c r="J18" t="s">
         <v>40</v>
       </c>
@@ -2718,7 +2722,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="10:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="10:11" x14ac:dyDescent="0.2">
       <c r="J19" t="s">
         <v>41</v>
       </c>
@@ -2726,7 +2730,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="10:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="10:11" x14ac:dyDescent="0.2">
       <c r="J20" t="s">
         <v>50</v>
       </c>
@@ -2734,7 +2738,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="10:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="10:11" x14ac:dyDescent="0.2">
       <c r="J21">
         <v>2</v>
       </c>
@@ -2742,7 +2746,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="10:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="10:11" x14ac:dyDescent="0.2">
       <c r="J22" t="s">
         <v>53</v>
       </c>
@@ -2759,14 +2763,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BBBD212-A842-4864-9B44-FE9AE1313599}">
   <dimension ref="A1:R22"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>1</v>
       </c>
@@ -2807,7 +2811,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2855,7 +2859,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2</v>
       </c>
@@ -2907,7 +2911,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>3</v>
       </c>
@@ -2952,7 +2956,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>4</v>
       </c>
@@ -2988,7 +2992,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>5</v>
       </c>
@@ -3024,7 +3028,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>6</v>
       </c>
@@ -3060,7 +3064,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>7</v>
       </c>
@@ -3096,7 +3100,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="J10" t="s">
         <v>44</v>
       </c>
@@ -3111,7 +3115,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="J11" t="s">
         <v>51</v>
       </c>
@@ -3126,7 +3130,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="J12" t="s">
         <v>37</v>
       </c>
@@ -3141,7 +3145,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>8</v>
       </c>
@@ -3177,7 +3181,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="J14">
         <v>1</v>
       </c>
@@ -3192,7 +3196,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="J15" t="s">
         <v>38</v>
       </c>
@@ -3207,7 +3211,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="J16" t="s">
         <v>52</v>
       </c>
@@ -3222,7 +3226,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>9</v>
       </c>
@@ -3258,7 +3262,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>10</v>
       </c>
@@ -3294,7 +3298,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J19" t="s">
         <v>41</v>
       </c>
@@ -3309,7 +3313,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>11</v>
       </c>
@@ -3345,7 +3349,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J21">
         <v>2</v>
       </c>
@@ -3360,7 +3364,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J22" t="s">
         <v>53</v>
       </c>
@@ -3383,14 +3387,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7267F07-2E02-4628-93AD-F735C6E325C1}">
   <dimension ref="A1:R22"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>1</v>
       </c>
@@ -3431,7 +3435,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
@@ -3479,7 +3483,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2</v>
       </c>
@@ -3531,7 +3535,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>3</v>
       </c>
@@ -3576,7 +3580,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>4</v>
       </c>
@@ -3612,7 +3616,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>5</v>
       </c>
@@ -3648,7 +3652,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>6</v>
       </c>
@@ -3684,7 +3688,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>7</v>
       </c>
@@ -3720,7 +3724,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>8</v>
       </c>
@@ -3756,7 +3760,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="J11" t="s">
         <v>51</v>
       </c>
@@ -3771,7 +3775,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="J12" t="s">
         <v>37</v>
       </c>
@@ -3786,7 +3790,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>9</v>
       </c>
@@ -3822,7 +3826,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>10</v>
       </c>
@@ -3858,7 +3862,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="J15" t="s">
         <v>38</v>
       </c>
@@ -3873,7 +3877,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="J16" t="s">
         <v>52</v>
       </c>
@@ -3888,7 +3892,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>11</v>
       </c>
@@ -3924,7 +3928,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>12</v>
       </c>
@@ -3960,7 +3964,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J19" t="s">
         <v>41</v>
       </c>
@@ -3975,7 +3979,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>13</v>
       </c>
@@ -4011,7 +4015,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>14</v>
       </c>
@@ -4047,7 +4051,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>15</v>
       </c>
@@ -4091,14 +4095,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60A64D70-CEA9-4F6F-AB92-E9B958DD131D}">
   <dimension ref="A1:R20"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>1</v>
       </c>
@@ -4139,7 +4143,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
@@ -4187,7 +4191,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2</v>
       </c>
@@ -4239,7 +4243,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>3</v>
       </c>
@@ -4284,7 +4288,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>4</v>
       </c>
@@ -4320,7 +4324,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>5</v>
       </c>
@@ -4356,7 +4360,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>6</v>
       </c>
@@ -4392,7 +4396,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="J9" t="s">
         <v>35</v>
       </c>
@@ -4407,7 +4411,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>7</v>
       </c>
@@ -4443,7 +4447,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>8</v>
       </c>
@@ -4482,7 +4486,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>9</v>
       </c>
@@ -4518,7 +4522,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>10</v>
       </c>
@@ -4554,7 +4558,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>11</v>
       </c>
@@ -4590,7 +4594,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>12</v>
       </c>
@@ -4626,7 +4630,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>13</v>
       </c>
@@ -4662,7 +4666,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>14</v>
       </c>
@@ -4698,7 +4702,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>15</v>
       </c>
@@ -4734,7 +4738,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>16</v>
       </c>
@@ -4770,7 +4774,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>17</v>
       </c>
@@ -4814,14 +4818,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B57BCD3D-EFFA-47F6-A031-A0E77D1E0022}">
   <dimension ref="A1:R19"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>1</v>
       </c>
@@ -4862,7 +4866,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
@@ -4910,7 +4914,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2</v>
       </c>
@@ -4962,7 +4966,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>3</v>
       </c>
@@ -5007,7 +5011,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>4</v>
       </c>
@@ -5043,7 +5047,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>5</v>
       </c>
@@ -5079,7 +5083,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>6</v>
       </c>
@@ -5115,7 +5119,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>7</v>
       </c>
@@ -5151,7 +5155,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>8</v>
       </c>
@@ -5187,7 +5191,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>9</v>
       </c>
@@ -5223,7 +5227,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>10</v>
       </c>
@@ -5259,7 +5263,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="J13" t="s">
         <v>51</v>
       </c>
@@ -5274,7 +5278,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="J14">
         <v>1</v>
       </c>
@@ -5289,7 +5293,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>11</v>
       </c>
@@ -5325,7 +5329,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>12</v>
       </c>
@@ -5361,7 +5365,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J17" t="s">
         <v>39</v>
       </c>
@@ -5376,7 +5380,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J18" t="s">
         <v>40</v>
       </c>
@@ -5391,7 +5395,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>13</v>
       </c>
@@ -5434,8 +5438,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009B0162F312A93D41AE706303C1572F17" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="66af2654134d243f62aac8e2b322f1d6">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8e1efd23-f4ba-42d2-85fd-6a510437bae6" xmlns:ns3="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2bc3adf68671d86faa9c37249f400344" ns2:_="" ns3:_="">
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="8e1efd23-f4ba-42d2-85fd-6a510437bae6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009B0162F312A93D41AE706303C1572F17" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d42a73f51a03135be35f4acb272f8cf1">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8e1efd23-f4ba-42d2-85fd-6a510437bae6" xmlns:ns3="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2ea21b36c10eaa86a5cb337ec7f4e0a6" ns2:_="" ns3:_="">
     <xsd:import namespace="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
     <xsd:import namespace="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
     <xsd:element name="properties">
@@ -5459,6 +5483,8 @@
                 <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -5533,6 +5559,16 @@
     <xsd:element name="MediaServiceSearchProperties" ma:index="23" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="24" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="25" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
@@ -5676,19 +5712,46 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6D48FD4C-247A-4C6F-B3F4-E10FE0F549E0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{656311BE-A32F-4883-81D7-E87C5D76E859}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C611BE04-F932-453D-B19B-D44103D0CF5E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C611BE04-F932-453D-B19B-D44103D0CF5E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6DCBF755-9035-4264-B566-07BF8202C15A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
+    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>